<commit_message>
requirements.txt and code fix for missing pandas import in Tumor_Volume_Excel.py.
</commit_message>
<xml_diff>
--- a/day02/T.V2.xlsx
+++ b/day02/T.V2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python\python-course-assignments\python-course-assignments\day02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CAD7FB5-A3CD-4C1C-823C-68F6A3272F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEF1D2C0-F203-4DA0-A55C-4546A7A29151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{60846883-93A2-42CD-91A5-DE46BEFCF260}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{60846883-93A2-42CD-91A5-DE46BEFCF260}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -124,7 +124,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -142,12 +142,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="32">
     <border>
@@ -587,7 +581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -715,8 +709,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -1202,10 +1194,10 @@
         <v>8</v>
       </c>
       <c r="D7" s="10"/>
-      <c r="E7" s="53">
+      <c r="E7" s="11">
         <v>6.88</v>
       </c>
-      <c r="F7" s="54">
+      <c r="F7" s="12">
         <v>5.7</v>
       </c>
       <c r="G7" s="13"/>

</xml_diff>